<commit_message>
Adding the most recent Seahorse data and moving a few old datasets to the `EXCLUDE` directories
</commit_message>
<xml_diff>
--- a/Excel_Data/PD220/XF Glycolytic Rate Assay  12.05.25  PD220,LV,Healthy with normalization-Quick View-Kinetic Graph.xlsx
+++ b/Excel_Data/PD220/XF Glycolytic Rate Assay  12.05.25  PD220,LV,Healthy with normalization-Quick View-Kinetic Graph.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardharris/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonardharris/PycharmProjects/FA_Metabolism/Excel_Data/PD220/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239CFE46-5E52-DE41-A4E8-2AFC79E22737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DBE373-150B-6348-8523-B8793E1A638F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1000" yWindow="1000" windowWidth="15000" windowHeight="10000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27460" yWindow="8180" windowWidth="15000" windowHeight="10000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kinetic Graph" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
     <t>Baseline</t>
   </si>
   <si>
-    <t>XF Glycolytic Rate Assay 12.5.2025 PD220,LV,Healthy with normalization</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -134,6 +131,9 @@
   </si>
   <si>
     <t>Healthy</t>
+  </si>
+  <si>
+    <t>XF Glycolytic Rate Assay 12.05.25 PD220,LV,Healthy with normalization</t>
   </si>
 </sst>
 </file>
@@ -626,18 +626,18 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
@@ -645,39 +645,39 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
@@ -687,10 +687,10 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -699,14 +699,14 @@
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O9" s="9"/>
       <c r="P9" s="9"/>
@@ -717,61 +717,61 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="B10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="5" t="s">
+      <c r="J10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="K10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="L10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="M10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="N10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="O10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="P10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="L10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="M10" s="5" t="s">
+      <c r="R10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="S10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="N10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="R10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="S10" s="3" t="s">
+      <c r="T10" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="T10" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>